<commit_message>
Auto update - 2026-04-04 15:53:52
</commit_message>
<xml_diff>
--- a/SaikumarMudam_Log Analtyic.xlsx
+++ b/SaikumarMudam_Log Analtyic.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91630\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E8E3CD-CB83-4644-8686-6182E855C28E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C6EDC8-8EC6-4D96-8E28-2FDF5B11564D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -370,7 +370,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="176">
   <si>
     <t>Planned Sprint</t>
   </si>
@@ -900,6 +900,54 @@
   <si>
     <t>Explore Dask and Ray</t>
   </si>
+  <si>
+    <t>Understanding the role of configuration files in project structure</t>
+  </si>
+  <si>
+    <t>Studied project architecture and implemented config module for better separation</t>
+  </si>
+  <si>
+    <t>Confusion in Dask concepts (Bag vs DataFrame processing)</t>
+  </si>
+  <si>
+    <t>Explored Dask documentation and tested sample examples for clarity</t>
+  </si>
+  <si>
+    <t>Difficulty in implementing Z-score calculation for anomaly detection</t>
+  </si>
+  <si>
+    <t>Revisited statistical concepts and validated implementation using sample data</t>
+  </si>
+  <si>
+    <t>Issue with SMTP email authentication while sending alerts</t>
+  </si>
+  <si>
+    <t>Configured Gmail App Password and enabled secure connection using starttls()</t>
+  </si>
+  <si>
+    <t>Errors in parsing and structuring raw log data</t>
+  </si>
+  <si>
+    <t>Debugged parsing logic and ensured correct schema mapping using metadata</t>
+  </si>
+  <si>
+    <t>Difficulty integrating Streamlit with backend pipeline</t>
+  </si>
+  <si>
+    <t>Refactored code to properly pass processed data into Streamlit dashboard</t>
+  </si>
+  <si>
+    <t>Plotly graphs not displaying correctly due to data format issues</t>
+  </si>
+  <si>
+    <t>Corrected DataFrame structure and verified visualization logic</t>
+  </si>
+  <si>
+    <t>Challenges in designing dashboard navigation (menu, dropdown, upload)</t>
+  </si>
+  <si>
+    <t>Implemented Streamlit UI components and structured dashboard layout</t>
+  </si>
 </sst>
 </file>
 
@@ -1332,7 +1380,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1492,26 +1540,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1545,6 +1573,29 @@
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3900,28 +3951,28 @@
       <c r="Z1" s="9"/>
     </row>
     <row r="2" spans="1:26" ht="45.75" customHeight="1">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="80" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="61" t="s">
+      <c r="C2" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="61" t="s">
+      <c r="D2" s="73" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="70" t="s">
+      <c r="E2" s="82" t="s">
         <v>49</v>
       </c>
-      <c r="F2" s="61" t="s">
+      <c r="F2" s="73" t="s">
         <v>50</v>
       </c>
-      <c r="G2" s="61" t="s">
+      <c r="G2" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="H2" s="61" t="s">
+      <c r="H2" s="73" t="s">
         <v>7</v>
       </c>
       <c r="I2" s="10" t="s">
@@ -3974,14 +4025,14 @@
       <c r="Z2" s="12"/>
     </row>
     <row r="3" spans="1:26" ht="30" customHeight="1">
-      <c r="A3" s="67"/>
-      <c r="B3" s="69"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
+      <c r="A3" s="79"/>
+      <c r="B3" s="81"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
       <c r="I3" s="13">
         <f t="shared" ref="I3:W3" si="0">SUM(I5:I802)</f>
         <v>82.5</v>
@@ -4047,31 +4098,31 @@
       <c r="Z3" s="12"/>
     </row>
     <row r="4" spans="1:26" ht="33.75" customHeight="1">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="75" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="64"/>
-      <c r="L4" s="64"/>
-      <c r="M4" s="64"/>
-      <c r="N4" s="64"/>
-      <c r="O4" s="64"/>
-      <c r="P4" s="64"/>
-      <c r="Q4" s="64"/>
-      <c r="R4" s="64"/>
-      <c r="S4" s="64"/>
-      <c r="T4" s="64"/>
-      <c r="U4" s="64"/>
-      <c r="V4" s="64"/>
-      <c r="W4" s="65"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
+      <c r="I4" s="76"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76"/>
+      <c r="L4" s="76"/>
+      <c r="M4" s="76"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="76"/>
+      <c r="Q4" s="76"/>
+      <c r="R4" s="76"/>
+      <c r="S4" s="76"/>
+      <c r="T4" s="76"/>
+      <c r="U4" s="76"/>
+      <c r="V4" s="76"/>
+      <c r="W4" s="77"/>
       <c r="X4" s="12"/>
       <c r="Y4" s="12"/>
       <c r="Z4" s="12"/>
@@ -4083,19 +4134,19 @@
       <c r="B5" s="15">
         <v>1</v>
       </c>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="77">
+      <c r="D5" s="67">
         <v>46055</v>
       </c>
-      <c r="E5" s="77">
+      <c r="E5" s="67">
         <v>46058</v>
       </c>
-      <c r="F5" s="76" t="s">
+      <c r="F5" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="G5" s="79" t="s">
+      <c r="G5" s="69" t="s">
         <v>136</v>
       </c>
       <c r="H5" s="53" t="s">
@@ -4157,19 +4208,19 @@
       <c r="B6" s="15">
         <v>2</v>
       </c>
-      <c r="C6" s="72" t="s">
+      <c r="C6" s="62" t="s">
         <v>146</v>
       </c>
-      <c r="D6" s="82">
+      <c r="D6" s="72">
         <v>46059</v>
       </c>
-      <c r="E6" s="82">
+      <c r="E6" s="72">
         <v>46063</v>
       </c>
-      <c r="F6" s="76" t="s">
+      <c r="F6" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="G6" s="79" t="s">
+      <c r="G6" s="69" t="s">
         <v>137</v>
       </c>
       <c r="H6" s="44" t="s">
@@ -4231,19 +4282,19 @@
       <c r="B7" s="15">
         <v>3</v>
       </c>
-      <c r="C7" s="72" t="s">
+      <c r="C7" s="62" t="s">
         <v>156</v>
       </c>
-      <c r="D7" s="82">
+      <c r="D7" s="72">
         <v>46066</v>
       </c>
-      <c r="E7" s="82">
+      <c r="E7" s="72">
         <v>46067</v>
       </c>
-      <c r="F7" s="76" t="s">
+      <c r="F7" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="G7" s="79" t="s">
+      <c r="G7" s="69" t="s">
         <v>152</v>
       </c>
       <c r="H7" s="44" t="s">
@@ -4305,19 +4356,19 @@
       <c r="B8" s="15">
         <v>4</v>
       </c>
-      <c r="C8" s="72" t="s">
+      <c r="C8" s="62" t="s">
         <v>138</v>
       </c>
-      <c r="D8" s="82">
+      <c r="D8" s="72">
         <v>46073</v>
       </c>
-      <c r="E8" s="82">
+      <c r="E8" s="72">
         <v>46075</v>
       </c>
-      <c r="F8" s="76" t="s">
+      <c r="F8" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="G8" s="79" t="s">
+      <c r="G8" s="69" t="s">
         <v>153</v>
       </c>
       <c r="H8" s="44" t="s">
@@ -4379,19 +4430,19 @@
       <c r="B9" s="15">
         <v>5</v>
       </c>
-      <c r="C9" s="72" t="s">
+      <c r="C9" s="62" t="s">
         <v>139</v>
       </c>
-      <c r="D9" s="82">
+      <c r="D9" s="72">
         <v>46077</v>
       </c>
-      <c r="E9" s="82">
+      <c r="E9" s="72">
         <v>46078</v>
       </c>
-      <c r="F9" s="76" t="s">
+      <c r="F9" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="G9" s="79" t="s">
+      <c r="G9" s="69" t="s">
         <v>153</v>
       </c>
       <c r="H9" s="44" t="s">
@@ -4453,19 +4504,19 @@
       <c r="B10" s="15">
         <v>6</v>
       </c>
-      <c r="C10" s="73" t="s">
+      <c r="C10" s="63" t="s">
         <v>140</v>
       </c>
-      <c r="D10" s="80">
+      <c r="D10" s="70">
         <v>46079</v>
       </c>
       <c r="E10" s="18">
         <v>46081</v>
       </c>
-      <c r="F10" s="75" t="s">
+      <c r="F10" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G10" s="79" t="s">
+      <c r="G10" s="69" t="s">
         <v>136</v>
       </c>
       <c r="H10" s="44" t="s">
@@ -4527,19 +4578,19 @@
       <c r="B11" s="15">
         <v>7</v>
       </c>
-      <c r="C11" s="73" t="s">
+      <c r="C11" s="63" t="s">
         <v>147</v>
       </c>
-      <c r="D11" s="81">
+      <c r="D11" s="71">
         <v>46084</v>
       </c>
       <c r="E11" s="18">
         <v>46085</v>
       </c>
-      <c r="F11" s="75" t="s">
+      <c r="F11" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G11" s="79" t="s">
+      <c r="G11" s="69" t="s">
         <v>136</v>
       </c>
       <c r="H11" s="44" t="s">
@@ -4601,19 +4652,19 @@
       <c r="B12" s="15">
         <v>8</v>
       </c>
-      <c r="C12" s="73" t="s">
+      <c r="C12" s="63" t="s">
         <v>141</v>
       </c>
-      <c r="D12" s="80">
+      <c r="D12" s="70">
         <v>46087</v>
       </c>
       <c r="E12" s="18">
         <v>46088</v>
       </c>
-      <c r="F12" s="75" t="s">
+      <c r="F12" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G12" s="79" t="s">
+      <c r="G12" s="69" t="s">
         <v>137</v>
       </c>
       <c r="H12" s="44" t="s">
@@ -4675,19 +4726,19 @@
       <c r="B13" s="15">
         <v>9</v>
       </c>
-      <c r="C13" s="73" t="s">
+      <c r="C13" s="63" t="s">
         <v>148</v>
       </c>
-      <c r="D13" s="80">
+      <c r="D13" s="70">
         <v>46090</v>
       </c>
       <c r="E13" s="18">
         <v>46091</v>
       </c>
-      <c r="F13" s="75" t="s">
+      <c r="F13" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G13" s="79" t="s">
+      <c r="G13" s="69" t="s">
         <v>153</v>
       </c>
       <c r="H13" s="44" t="s">
@@ -4749,19 +4800,19 @@
       <c r="B14" s="15">
         <v>10</v>
       </c>
-      <c r="C14" s="73" t="s">
+      <c r="C14" s="63" t="s">
         <v>149</v>
       </c>
-      <c r="D14" s="80">
+      <c r="D14" s="70">
         <v>46092</v>
       </c>
       <c r="E14" s="18">
         <v>46092</v>
       </c>
-      <c r="F14" s="75" t="s">
+      <c r="F14" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G14" s="79" t="s">
+      <c r="G14" s="69" t="s">
         <v>137</v>
       </c>
       <c r="H14" s="44" t="s">
@@ -4821,19 +4872,19 @@
       <c r="B15" s="15">
         <v>11</v>
       </c>
-      <c r="C15" s="73" t="s">
+      <c r="C15" s="63" t="s">
         <v>159</v>
       </c>
-      <c r="D15" s="80">
+      <c r="D15" s="70">
         <v>46094</v>
       </c>
       <c r="E15" s="18">
         <v>46095</v>
       </c>
-      <c r="F15" s="75" t="s">
+      <c r="F15" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G15" s="79" t="s">
+      <c r="G15" s="69" t="s">
         <v>153</v>
       </c>
       <c r="H15" s="44" t="s">
@@ -4889,25 +4940,25 @@
       <c r="Z15" s="9"/>
     </row>
     <row r="16" spans="1:26" ht="36.75" customHeight="1">
-      <c r="A16" s="71" t="s">
+      <c r="A16" s="61" t="s">
         <v>9</v>
       </c>
       <c r="B16" s="15">
         <v>12</v>
       </c>
-      <c r="C16" s="73" t="s">
+      <c r="C16" s="63" t="s">
         <v>150</v>
       </c>
-      <c r="D16" s="80">
+      <c r="D16" s="70">
         <v>46097</v>
       </c>
       <c r="E16" s="18">
         <v>46098</v>
       </c>
-      <c r="F16" s="75" t="s">
+      <c r="F16" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G16" s="79" t="s">
+      <c r="G16" s="69" t="s">
         <v>153</v>
       </c>
       <c r="H16" s="44" t="s">
@@ -4961,25 +5012,25 @@
       <c r="Z16" s="9"/>
     </row>
     <row r="17" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A17" s="71" t="s">
+      <c r="A17" s="61" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="15">
         <v>13</v>
       </c>
-      <c r="C17" s="73" t="s">
+      <c r="C17" s="63" t="s">
         <v>142</v>
       </c>
-      <c r="D17" s="80">
+      <c r="D17" s="70">
         <v>46100</v>
       </c>
       <c r="E17" s="18">
         <v>46100</v>
       </c>
-      <c r="F17" s="75" t="s">
+      <c r="F17" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G17" s="79" t="s">
+      <c r="G17" s="69" t="s">
         <v>136</v>
       </c>
       <c r="H17" s="44" t="s">
@@ -5041,19 +5092,19 @@
       <c r="B18" s="15">
         <v>14</v>
       </c>
-      <c r="C18" s="73" t="s">
+      <c r="C18" s="63" t="s">
         <v>151</v>
       </c>
-      <c r="D18" s="80">
+      <c r="D18" s="70">
         <v>46101</v>
       </c>
       <c r="E18" s="18">
         <v>46102</v>
       </c>
-      <c r="F18" s="75" t="s">
+      <c r="F18" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G18" s="79" t="s">
+      <c r="G18" s="69" t="s">
         <v>137</v>
       </c>
       <c r="H18" s="44" t="s">
@@ -5115,19 +5166,19 @@
       <c r="B19" s="15">
         <v>15</v>
       </c>
-      <c r="C19" s="73" t="s">
+      <c r="C19" s="63" t="s">
         <v>143</v>
       </c>
-      <c r="D19" s="80">
+      <c r="D19" s="70">
         <v>46103</v>
       </c>
       <c r="E19" s="18">
         <v>46103</v>
       </c>
-      <c r="F19" s="75" t="s">
+      <c r="F19" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G19" s="79" t="s">
+      <c r="G19" s="69" t="s">
         <v>153</v>
       </c>
       <c r="H19" s="44" t="s">
@@ -5189,19 +5240,19 @@
       <c r="B20" s="15">
         <v>16</v>
       </c>
-      <c r="C20" s="73" t="s">
+      <c r="C20" s="63" t="s">
         <v>157</v>
       </c>
-      <c r="D20" s="80">
+      <c r="D20" s="70">
         <v>46104</v>
       </c>
       <c r="E20" s="18">
         <v>46104</v>
       </c>
-      <c r="F20" s="75" t="s">
+      <c r="F20" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G20" s="79" t="s">
+      <c r="G20" s="69" t="s">
         <v>153</v>
       </c>
       <c r="H20" s="44" t="s">
@@ -5263,19 +5314,19 @@
       <c r="B21" s="15">
         <v>17</v>
       </c>
-      <c r="C21" s="73" t="s">
+      <c r="C21" s="63" t="s">
         <v>144</v>
       </c>
-      <c r="D21" s="80">
+      <c r="D21" s="70">
         <v>46105</v>
       </c>
       <c r="E21" s="18">
         <v>46105</v>
       </c>
-      <c r="F21" s="75" t="s">
+      <c r="F21" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G21" s="79" t="s">
+      <c r="G21" s="69" t="s">
         <v>154</v>
       </c>
       <c r="H21" s="44" t="s">
@@ -5337,19 +5388,19 @@
       <c r="B22" s="15">
         <v>18</v>
       </c>
-      <c r="C22" s="73" t="s">
+      <c r="C22" s="63" t="s">
         <v>158</v>
       </c>
-      <c r="D22" s="80">
+      <c r="D22" s="70">
         <v>46077</v>
       </c>
-      <c r="E22" s="78">
+      <c r="E22" s="68">
         <v>46106</v>
       </c>
-      <c r="F22" s="75" t="s">
+      <c r="F22" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="79" t="s">
+      <c r="G22" s="69" t="s">
         <v>155</v>
       </c>
       <c r="H22" s="44" t="s">
@@ -5409,19 +5460,19 @@
       <c r="B23" s="15">
         <v>19</v>
       </c>
-      <c r="C23" s="73" t="s">
+      <c r="C23" s="63" t="s">
         <v>145</v>
       </c>
-      <c r="D23" s="80">
+      <c r="D23" s="70">
         <v>46107</v>
       </c>
       <c r="E23" s="18">
         <v>46108</v>
       </c>
-      <c r="F23" s="75" t="s">
+      <c r="F23" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="G23" s="79" t="s">
+      <c r="G23" s="69" t="s">
         <v>136</v>
       </c>
       <c r="H23" s="44" t="s">
@@ -16105,52 +16156,116 @@
       <c r="G1" s="35"/>
     </row>
     <row r="2" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A2" s="36"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
+      <c r="A2" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="36">
+        <v>1</v>
+      </c>
+      <c r="C2" s="83" t="s">
+        <v>160</v>
+      </c>
+      <c r="D2" s="83" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A3" s="36"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
+      <c r="A3" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="36">
+        <v>2</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>162</v>
+      </c>
+      <c r="D3" s="83" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
+      <c r="A4" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="36">
+        <v>3</v>
+      </c>
+      <c r="C4" s="83" t="s">
+        <v>164</v>
+      </c>
+      <c r="D4" s="83" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A5" s="36"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
+      <c r="A5" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="36">
+        <v>4</v>
+      </c>
+      <c r="C5" s="83" t="s">
+        <v>166</v>
+      </c>
+      <c r="D5" s="83" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A6" s="36"/>
-      <c r="B6" s="36"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
+      <c r="A6" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="36">
+        <v>5</v>
+      </c>
+      <c r="C6" s="83" t="s">
+        <v>168</v>
+      </c>
+      <c r="D6" s="83" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A7" s="36"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
+      <c r="A7" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="36">
+        <v>6</v>
+      </c>
+      <c r="C7" s="83" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7" s="83" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A8" s="36"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
+      <c r="A8" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="36">
+        <v>7</v>
+      </c>
+      <c r="C8" s="83" t="s">
+        <v>172</v>
+      </c>
+      <c r="D8" s="83" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="9" spans="1:7" ht="12.75" customHeight="1">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
+      <c r="A9" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="36">
+        <v>8</v>
+      </c>
+      <c r="C9" s="83" t="s">
+        <v>174</v>
+      </c>
+      <c r="D9" s="83" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="10" spans="1:7" ht="12.75" customHeight="1"/>
     <row r="11" spans="1:7" ht="12.75" customHeight="1"/>
@@ -17144,6 +17259,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
+  <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>

</xml_diff>